<commit_message>
FIXED: 58 formulas properly inserted into ORION template
</commit_message>
<xml_diff>
--- a/PROJECTS/ORION/ORION_LIGHTING_FILLED.xlsx
+++ b/PROJECTS/ORION/ORION_LIGHTING_FILLED.xlsx
@@ -708,19 +708,25 @@
       <c r="A13" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="B13" s="12"/>
+      <c r="B13">
+        <f>Sheet2!B17+SUM(Sheet2!C17:H17)</f>
+      </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" s="13" t="s">
         <v>42</v>
       </c>
-      <c r="B14" s="14"/>
+      <c r="B14">
+        <f>IRR(Sheet2!B13:H13)</f>
+      </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15" s="13" t="s">
         <v>43</v>
       </c>
-      <c r="B15" s="15"/>
+      <c r="B15">
+        <f>(B13+Sheet1!$B$2)/Sheet1!$B$2</f>
+      </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16" s="13" t="s">
@@ -780,100 +786,200 @@
       <c r="A3" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C3" s="4"/>
-      <c r="D3" s="4"/>
-      <c r="E3" s="4"/>
-      <c r="F3" s="4"/>
-      <c r="G3" s="4"/>
-      <c r="H3" s="4"/>
+      <c r="C3">
+        <f>Sheet1!$B$9</f>
+      </c>
+      <c r="D3">
+        <f>C3*(1+Sheet1!$B$10)</f>
+      </c>
+      <c r="E3">
+        <f>D3*(1+Sheet1!$B$10)</f>
+      </c>
+      <c r="F3">
+        <f>E3*(1+Sheet1!$B$10)</f>
+      </c>
+      <c r="G3">
+        <f>F3*(1+Sheet1!$B$10)</f>
+      </c>
+      <c r="H3">
+        <f>G3*(1+Sheet1!$B$10)</f>
+      </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C4" s="4"/>
-      <c r="D4" s="4"/>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4"/>
-      <c r="G4" s="4"/>
-      <c r="H4" s="4"/>
+      <c r="C4">
+        <f>C3*Sheet1!$B$11</f>
+      </c>
+      <c r="D4">
+        <f>D3*Sheet1!$B$11</f>
+      </c>
+      <c r="E4">
+        <f>E3*Sheet1!$B$11</f>
+      </c>
+      <c r="F4">
+        <f>F3*Sheet1!$B$11</f>
+      </c>
+      <c r="G4">
+        <f>G3*Sheet1!$B$11</f>
+      </c>
+      <c r="H4">
+        <f>G3*Sheet1!$B$11</f>
+      </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
-      <c r="E5" s="4"/>
-      <c r="F5" s="4"/>
-      <c r="G5" s="4"/>
-      <c r="H5" s="4"/>
+      <c r="C5">
+        <f>(Sheet1!$B$2-Sheet1!$B$5)/Sheet1!$B$6</f>
+      </c>
+      <c r="D5">
+        <f>(Sheet1!$B$2-Sheet1!$B$5)/Sheet1!$B$6</f>
+      </c>
+      <c r="E5">
+        <f>(Sheet1!$B$2-Sheet1!$B$5)/Sheet1!$B$6</f>
+      </c>
+      <c r="F5">
+        <f>(Sheet1!$B$2-Sheet1!$B$5)/Sheet1!$B$6</f>
+      </c>
+      <c r="G5">
+        <f>(Sheet1!$B$2-Sheet1!$B$5)/Sheet1!$B$6</f>
+      </c>
+      <c r="H5">
+        <f>(Sheet1!$B$2-Sheet1!$B$5)/Sheet1!$B$6</f>
+      </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>21</v>
       </c>
       <c r="B6" s="4"/>
-      <c r="C6" s="4"/>
-      <c r="D6" s="4"/>
-      <c r="E6" s="4"/>
-      <c r="F6" s="4"/>
-      <c r="G6" s="4"/>
+      <c r="C6">
+        <f>C3+C4+C5</f>
+      </c>
+      <c r="D6">
+        <f>D3+D4+D5</f>
+      </c>
+      <c r="E6">
+        <f>E3+E4+E5</f>
+      </c>
+      <c r="F6">
+        <f>F3+F4+F5</f>
+      </c>
+      <c r="G6">
+        <f>G3+G4+G5</f>
+      </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>22</v>
       </c>
       <c r="B7" s="4"/>
-      <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
-      <c r="E7" s="4"/>
-      <c r="F7" s="4"/>
-      <c r="G7" s="4"/>
+      <c r="C7">
+        <f>C6*Sheet1!$B$7</f>
+      </c>
+      <c r="D7">
+        <f>D6*Sheet1!$B$7</f>
+      </c>
+      <c r="E7">
+        <f>E6*Sheet1!$B$7</f>
+      </c>
+      <c r="F7">
+        <f>F6*Sheet1!$B$7</f>
+      </c>
+      <c r="G7">
+        <f>G6*Sheet1!$B$7</f>
+      </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>23</v>
       </c>
       <c r="B8" s="1"/>
-      <c r="C8" s="6"/>
-      <c r="D8" s="6"/>
-      <c r="E8" s="6"/>
-      <c r="F8" s="6"/>
-      <c r="G8" s="6"/>
+      <c r="C8">
+        <f>C6+C7</f>
+      </c>
+      <c r="D8">
+        <f>D6+D7</f>
+      </c>
+      <c r="E8">
+        <f>E6+E7</f>
+      </c>
+      <c r="F8">
+        <f>F6+F7</f>
+      </c>
+      <c r="G8">
+        <f>G6+G7</f>
+      </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>24</v>
       </c>
       <c r="B9" s="4"/>
-      <c r="C9" s="4"/>
-      <c r="D9" s="4"/>
-      <c r="E9" s="4"/>
-      <c r="F9" s="4"/>
-      <c r="G9" s="4"/>
+      <c r="C9">
+        <f>C5</f>
+      </c>
+      <c r="D9">
+        <f>D5</f>
+      </c>
+      <c r="E9">
+        <f>E5</f>
+      </c>
+      <c r="F9">
+        <f>F5</f>
+      </c>
+      <c r="G9">
+        <f>G5</f>
+      </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B10" s="4"/>
-      <c r="C10" s="4"/>
-      <c r="D10" s="4"/>
-      <c r="E10" s="4"/>
-      <c r="F10" s="4"/>
-      <c r="G10" s="4"/>
+      <c r="B10">
+        <f>-Sheet1!$B$2</f>
+      </c>
+      <c r="C10">
+        <f>0</f>
+      </c>
+      <c r="D10">
+        <f>0</f>
+      </c>
+      <c r="E10">
+        <f>0</f>
+      </c>
+      <c r="F10">
+        <f>0</f>
+      </c>
+      <c r="G10">
+        <f>0</f>
+      </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="B11" s="4"/>
-      <c r="C11" s="4"/>
-      <c r="D11" s="4"/>
-      <c r="E11" s="4"/>
-      <c r="F11" s="4"/>
-      <c r="G11" s="4"/>
+      <c r="B11">
+        <f>0</f>
+      </c>
+      <c r="C11">
+        <f>-C3*Sheet1!$B$12</f>
+      </c>
+      <c r="D11">
+        <f>-(D3-C3)*Sheet1!$B$12</f>
+      </c>
+      <c r="E11">
+        <f>-(E3-D3)*Sheet1!$B$12</f>
+      </c>
+      <c r="F11">
+        <f>-(F3-E3)*Sheet1!$B$12</f>
+      </c>
+      <c r="G11">
+        <f>-(G3-F3)*Sheet1!$B$12</f>
+      </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A12" s="10" t="s">
@@ -885,12 +991,24 @@
       <c r="A13" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B13" s="6"/>
-      <c r="C13" s="6"/>
-      <c r="D13" s="6"/>
-      <c r="E13" s="6"/>
-      <c r="F13" s="6"/>
-      <c r="G13" s="6"/>
+      <c r="B13">
+        <f>B8+B9+B10+B11</f>
+      </c>
+      <c r="C13">
+        <f>C8+C9+C10+C11</f>
+      </c>
+      <c r="D13">
+        <f>D8+D9+D10+D11</f>
+      </c>
+      <c r="E13">
+        <f>E8+E9+E10+E11</f>
+      </c>
+      <c r="F13">
+        <f>F8+F9+F10+F11</f>
+      </c>
+      <c r="G13">
+        <f>G8+G9+G10+G11</f>
+      </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.35">
       <c r="C14" s="4"/>
@@ -903,13 +1021,17 @@
       <c r="A15" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B15" s="9"/>
+      <c r="B15">
+        <f>1</f>
+      </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="B17" s="6"/>
+      <c r="B17">
+        <f>B13*B15</f>
+      </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">

</xml_diff>

<commit_message>
Properly filled ORION template with 55 formulas
</commit_message>
<xml_diff>
--- a/PROJECTS/ORION/ORION_LIGHTING_FILLED.xlsx
+++ b/PROJECTS/ORION/ORION_LIGHTING_FILLED.xlsx
@@ -709,7 +709,8 @@
         <v>41</v>
       </c>
       <c r="B13">
-        <f>Sheet2!B17+SUM(Sheet2!C17:H17)</f>
+        <f>Sheet2!B17+SUM(Sheet2!C17:G17)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.35">
@@ -717,7 +718,8 @@
         <v>42</v>
       </c>
       <c r="B14">
-        <f>IRR(Sheet2!B13:H13)</f>
+        <f>IRR(Sheet2!B13:G13)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.35">
@@ -726,6 +728,7 @@
       </c>
       <c r="B15">
         <f>(B13+Sheet1!$B$2)/Sheet1!$B$2</f>
+        <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.35">
@@ -788,22 +791,25 @@
       </c>
       <c r="C3">
         <f>Sheet1!$B$9</f>
+        <v>0</v>
       </c>
       <c r="D3">
         <f>C3*(1+Sheet1!$B$10)</f>
+        <v>0</v>
       </c>
       <c r="E3">
         <f>D3*(1+Sheet1!$B$10)</f>
+        <v>0</v>
       </c>
       <c r="F3">
         <f>E3*(1+Sheet1!$B$10)</f>
+        <v>0</v>
       </c>
       <c r="G3">
         <f>F3*(1+Sheet1!$B$10)</f>
-      </c>
-      <c r="H3">
-        <f>G3*(1+Sheet1!$B$10)</f>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="H3" s="4"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
@@ -811,45 +817,51 @@
       </c>
       <c r="C4">
         <f>C3*Sheet1!$B$11</f>
+        <v>0</v>
       </c>
       <c r="D4">
         <f>D3*Sheet1!$B$11</f>
+        <v>0</v>
       </c>
       <c r="E4">
         <f>E3*Sheet1!$B$11</f>
+        <v>0</v>
       </c>
       <c r="F4">
         <f>F3*Sheet1!$B$11</f>
+        <v>0</v>
       </c>
       <c r="G4">
         <f>G3*Sheet1!$B$11</f>
-      </c>
-      <c r="H4">
-        <f>G3*Sheet1!$B$11</f>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="H4" s="4"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
       <c r="C5">
-        <f>(Sheet1!$B$2-Sheet1!$B$5)/Sheet1!$B$6</f>
+        <f>(Sheet1!$B$2-Sheet1!$B$3)/Sheet1!$B$4</f>
+        <v>0</v>
       </c>
       <c r="D5">
-        <f>(Sheet1!$B$2-Sheet1!$B$5)/Sheet1!$B$6</f>
+        <f>(Sheet1!$B$2-Sheet1!$B$3)/Sheet1!$B$4</f>
+        <v>0</v>
       </c>
       <c r="E5">
-        <f>(Sheet1!$B$2-Sheet1!$B$5)/Sheet1!$B$6</f>
+        <f>(Sheet1!$B$2-Sheet1!$B$3)/Sheet1!$B$4</f>
+        <v>0</v>
       </c>
       <c r="F5">
-        <f>(Sheet1!$B$2-Sheet1!$B$5)/Sheet1!$B$6</f>
+        <f>(Sheet1!$B$2-Sheet1!$B$3)/Sheet1!$B$4</f>
+        <v>0</v>
       </c>
       <c r="G5">
-        <f>(Sheet1!$B$2-Sheet1!$B$5)/Sheet1!$B$6</f>
-      </c>
-      <c r="H5">
-        <f>(Sheet1!$B$2-Sheet1!$B$5)/Sheet1!$B$6</f>
-      </c>
+        <f>(Sheet1!$B$2-Sheet1!$B$3)/Sheet1!$B$4</f>
+        <v>0</v>
+      </c>
+      <c r="H5" s="4"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
@@ -858,18 +870,23 @@
       <c r="B6" s="4"/>
       <c r="C6">
         <f>C3+C4+C5</f>
+        <v>0</v>
       </c>
       <c r="D6">
         <f>D3+D4+D5</f>
+        <v>0</v>
       </c>
       <c r="E6">
         <f>E3+E4+E5</f>
+        <v>0</v>
       </c>
       <c r="F6">
         <f>F3+F4+F5</f>
+        <v>0</v>
       </c>
       <c r="G6">
         <f>G3+G4+G5</f>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.35">
@@ -878,19 +895,24 @@
       </c>
       <c r="B7" s="4"/>
       <c r="C7">
-        <f>C6*Sheet1!$B$7</f>
+        <f>C6*Sheet1!$B$5</f>
+        <v>0</v>
       </c>
       <c r="D7">
-        <f>D6*Sheet1!$B$7</f>
+        <f>D6*Sheet1!$B$5</f>
+        <v>0</v>
       </c>
       <c r="E7">
-        <f>E6*Sheet1!$B$7</f>
+        <f>E6*Sheet1!$B$5</f>
+        <v>0</v>
       </c>
       <c r="F7">
-        <f>F6*Sheet1!$B$7</f>
+        <f>F6*Sheet1!$B$5</f>
+        <v>0</v>
       </c>
       <c r="G7">
-        <f>G6*Sheet1!$B$7</f>
+        <f>G6*Sheet1!$B$5</f>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.35">
@@ -900,18 +922,23 @@
       <c r="B8" s="1"/>
       <c r="C8">
         <f>C6+C7</f>
+        <v>0</v>
       </c>
       <c r="D8">
         <f>D6+D7</f>
+        <v>0</v>
       </c>
       <c r="E8">
         <f>E6+E7</f>
+        <v>0</v>
       </c>
       <c r="F8">
         <f>F6+F7</f>
+        <v>0</v>
       </c>
       <c r="G8">
         <f>G6+G7</f>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.35">
@@ -921,18 +948,23 @@
       <c r="B9" s="4"/>
       <c r="C9">
         <f>C5</f>
+        <v>0</v>
       </c>
       <c r="D9">
         <f>D5</f>
+        <v>0</v>
       </c>
       <c r="E9">
         <f>E5</f>
+        <v>0</v>
       </c>
       <c r="F9">
         <f>F5</f>
+        <v>0</v>
       </c>
       <c r="G9">
         <f>G5</f>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.35">
@@ -941,21 +973,27 @@
       </c>
       <c r="B10">
         <f>-Sheet1!$B$2</f>
+        <v>0</v>
       </c>
       <c r="C10">
         <f>0</f>
+        <v>0</v>
       </c>
       <c r="D10">
         <f>0</f>
+        <v>0</v>
       </c>
       <c r="E10">
         <f>0</f>
+        <v>0</v>
       </c>
       <c r="F10">
         <f>0</f>
+        <v>0</v>
       </c>
       <c r="G10">
         <f>0</f>
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.35">
@@ -964,21 +1002,27 @@
       </c>
       <c r="B11">
         <f>0</f>
+        <v>0</v>
       </c>
       <c r="C11">
-        <f>-C3*Sheet1!$B$12</f>
+        <f>-C3*Sheet1!$B$10</f>
+        <v>0</v>
       </c>
       <c r="D11">
-        <f>-(D3-C3)*Sheet1!$B$12</f>
+        <f>-(D3-C3)*Sheet1!$B$10</f>
+        <v>0</v>
       </c>
       <c r="E11">
-        <f>-(E3-D3)*Sheet1!$B$12</f>
+        <f>-(E3-D3)*Sheet1!$B$10</f>
+        <v>0</v>
       </c>
       <c r="F11">
-        <f>-(F3-E3)*Sheet1!$B$12</f>
+        <f>-(F3-E3)*Sheet1!$B$10</f>
+        <v>0</v>
       </c>
       <c r="G11">
-        <f>-(G3-F3)*Sheet1!$B$12</f>
+        <f>-(G3-F3)*Sheet1!$B$10</f>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.35">
@@ -993,21 +1037,27 @@
       </c>
       <c r="B13">
         <f>B8+B9+B10+B11</f>
+        <v>0</v>
       </c>
       <c r="C13">
         <f>C8+C9+C10+C11</f>
+        <v>0</v>
       </c>
       <c r="D13">
         <f>D8+D9+D10+D11</f>
+        <v>0</v>
       </c>
       <c r="E13">
         <f>E8+E9+E10+E11</f>
+        <v>0</v>
       </c>
       <c r="F13">
         <f>F8+F9+F10+F11</f>
+        <v>0</v>
       </c>
       <c r="G13">
         <f>G8+G9+G10+G11</f>
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.35">
@@ -1023,6 +1073,7 @@
       </c>
       <c r="B15">
         <f>1</f>
+        <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.35">
@@ -1031,6 +1082,7 @@
       </c>
       <c r="B17">
         <f>B13*B15</f>
+        <v>0</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.35">

</xml_diff>